<commit_message>
Actualización: Agregar Club America a la base de datos
</commit_message>
<xml_diff>
--- a/lmi temp 10.xlsx
+++ b/lmi temp 10.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82585704-B76D-4A8C-A14A-C40E5CE159E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71D6320-9531-420A-A25E-683CDE7D6816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1907" uniqueCount="968">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1960" uniqueCount="1020">
   <si>
     <t>Inter_de_Milan</t>
   </si>
@@ -3002,6 +3002,162 @@
   </si>
   <si>
     <t>DC Carlos Espi</t>
+  </si>
+  <si>
+    <t>Club_America</t>
+  </si>
+  <si>
+    <t>Yann Sommer</t>
+  </si>
+  <si>
+    <t>Luke Shaw</t>
+  </si>
+  <si>
+    <t>Alessandro Deiola</t>
+  </si>
+  <si>
+    <t>Amir Rrahmani</t>
+  </si>
+  <si>
+    <t>Joshua Kimmich</t>
+  </si>
+  <si>
+    <t>Sergio Busquets</t>
+  </si>
+  <si>
+    <t>Seko Fofana</t>
+  </si>
+  <si>
+    <t>Lee Jae-sung</t>
+  </si>
+  <si>
+    <t>Rodrigo Garro</t>
+  </si>
+  <si>
+    <t>Gerard Moreno</t>
+  </si>
+  <si>
+    <t>Alessandro Del Piero</t>
+  </si>
+  <si>
+    <t>Lucas Perri</t>
+  </si>
+  <si>
+    <t>Sebastián Cáceres</t>
+  </si>
+  <si>
+    <t>Miguel Layún</t>
+  </si>
+  <si>
+    <t>Lucas Digne</t>
+  </si>
+  <si>
+    <t>Ross Barkley</t>
+  </si>
+  <si>
+    <t>Yacine Adli</t>
+  </si>
+  <si>
+    <t>Álvaro Fidalgo</t>
+  </si>
+  <si>
+    <t>Tommaso Baldanzi</t>
+  </si>
+  <si>
+    <t>Olivier Giroud</t>
+  </si>
+  <si>
+    <t>Florian Thauvin</t>
+  </si>
+  <si>
+    <t>Ciro Immobile</t>
+  </si>
+  <si>
+    <t>Gabriel Barbosa</t>
+  </si>
+  <si>
+    <t>Club America</t>
+  </si>
+  <si>
+    <t>PT Yann Sommer</t>
+  </si>
+  <si>
+    <t>LI Luke Shaw</t>
+  </si>
+  <si>
+    <t>MC Alessandro Deiola</t>
+  </si>
+  <si>
+    <t>CT Amir Rrahmani</t>
+  </si>
+  <si>
+    <t>MCD Joshua Kimmich</t>
+  </si>
+  <si>
+    <t>MCD Sergio Busquets</t>
+  </si>
+  <si>
+    <t>MC Seko Fofana</t>
+  </si>
+  <si>
+    <t>MP Lee Jae-sung</t>
+  </si>
+  <si>
+    <t>MP Rodrigo Garro</t>
+  </si>
+  <si>
+    <t>DC Gerard Moreno</t>
+  </si>
+  <si>
+    <t>DC Alessandro Del Piero</t>
+  </si>
+  <si>
+    <t>PT Lucas Perri</t>
+  </si>
+  <si>
+    <t>CT Sebastián Cáceres</t>
+  </si>
+  <si>
+    <t>LD Miguel Layún</t>
+  </si>
+  <si>
+    <t>LI Lucas Digne</t>
+  </si>
+  <si>
+    <t>MC Ross Barkley</t>
+  </si>
+  <si>
+    <t>MC Yacine Adli</t>
+  </si>
+  <si>
+    <t>MC Álvaro Fidalgo</t>
+  </si>
+  <si>
+    <t>MP Tommaso Baldanzi</t>
+  </si>
+  <si>
+    <t>DC Olivier Giroud</t>
+  </si>
+  <si>
+    <t>ED Florian Thauvin</t>
+  </si>
+  <si>
+    <t>DC Ciro Immobile</t>
+  </si>
+  <si>
+    <t>DC Gabriel Barbosa</t>
+  </si>
+  <si>
+    <t>AME</t>
+  </si>
+  <si>
+    <t>Estadio Banorte</t>
+  </si>
+  <si>
+    <t>Jose Diaz</t>
+  </si>
+  <si>
+    <t>Logos Equipos/clubamerica.png</t>
   </si>
 </sst>
 </file>
@@ -3072,7 +3228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3091,6 +3247,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10670,29 +10829,30 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.77734375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.77734375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.109375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -10744,8 +10904,11 @@
       <c r="Q1" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R1" s="8" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
@@ -10797,8 +10960,11 @@
       <c r="Q2" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R2" s="3" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>32</v>
       </c>
@@ -10850,8 +11016,11 @@
       <c r="Q3" s="3" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R3" s="3" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>48</v>
       </c>
@@ -10903,8 +11072,11 @@
       <c r="Q4" s="3" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R4" s="3" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>64</v>
       </c>
@@ -10956,8 +11128,11 @@
       <c r="Q5" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R5" s="3" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>80</v>
       </c>
@@ -11009,8 +11184,11 @@
       <c r="Q6" s="3" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R6" s="3" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>96</v>
       </c>
@@ -11062,8 +11240,11 @@
       <c r="Q7" s="3" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R7" s="3" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>112</v>
       </c>
@@ -11115,8 +11296,11 @@
       <c r="Q8" s="3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R8" s="3" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>128</v>
       </c>
@@ -11168,8 +11352,11 @@
       <c r="Q9" s="3" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R9" s="3" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>144</v>
       </c>
@@ -11221,8 +11408,11 @@
       <c r="Q10" s="3" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R10" s="3" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>159</v>
       </c>
@@ -11274,8 +11464,11 @@
       <c r="Q11" s="3" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R11" s="3" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>175</v>
       </c>
@@ -11327,8 +11520,11 @@
       <c r="Q12" s="3" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R12" s="3" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>191</v>
       </c>
@@ -11380,8 +11576,11 @@
       <c r="Q13" s="3" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R13" s="3" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>207</v>
       </c>
@@ -11433,8 +11632,11 @@
       <c r="Q14" s="3" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R14" s="3" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>223</v>
       </c>
@@ -11486,8 +11688,11 @@
       <c r="Q15" s="3" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R15" s="3" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>239</v>
       </c>
@@ -11539,8 +11744,11 @@
       <c r="Q16" s="3" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R16" s="3" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>255</v>
       </c>
@@ -11592,8 +11800,11 @@
       <c r="Q17" s="3" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R17" s="3" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>271</v>
       </c>
@@ -11645,8 +11856,11 @@
       <c r="Q18" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R18" s="3" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>287</v>
       </c>
@@ -11698,8 +11912,11 @@
       <c r="Q19" s="3" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R19" s="3" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>302</v>
       </c>
@@ -11751,8 +11968,11 @@
       <c r="Q20" s="3" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R20" s="3" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>318</v>
       </c>
@@ -11804,8 +12024,11 @@
       <c r="Q21" s="3" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R21" s="3" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>334</v>
       </c>
@@ -11857,8 +12080,11 @@
       <c r="Q22" s="3" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R22" s="3" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>350</v>
       </c>
@@ -11910,8 +12136,11 @@
       <c r="Q23" s="3" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R23" s="3" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>366</v>
       </c>
@@ -11962,6 +12191,9 @@
       </c>
       <c r="Q24" s="3" t="s">
         <v>381</v>
+      </c>
+      <c r="R24" s="3" t="s">
+        <v>991</v>
       </c>
     </row>
   </sheetData>
@@ -12046,7 +12278,9 @@
       <c r="Q1" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="R1" s="3"/>
+      <c r="R1" s="3" t="s">
+        <v>992</v>
+      </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -12100,7 +12334,9 @@
       <c r="Q2" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="R2" s="3"/>
+      <c r="R2" s="3" t="s">
+        <v>993</v>
+      </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -12154,7 +12390,9 @@
       <c r="Q3" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="R3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>994</v>
+      </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
@@ -12208,7 +12446,9 @@
       <c r="Q4" s="3" t="s">
         <v>473</v>
       </c>
-      <c r="R4" s="3"/>
+      <c r="R4" s="3" t="s">
+        <v>995</v>
+      </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -12262,7 +12502,9 @@
       <c r="Q5" s="3" t="s">
         <v>489</v>
       </c>
-      <c r="R5" s="3"/>
+      <c r="R5" s="3" t="s">
+        <v>996</v>
+      </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -12316,7 +12558,9 @@
       <c r="Q6" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="R6" s="3"/>
+      <c r="R6" s="3" t="s">
+        <v>997</v>
+      </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -12370,7 +12614,9 @@
       <c r="Q7" s="3" t="s">
         <v>521</v>
       </c>
-      <c r="R7" s="3"/>
+      <c r="R7" s="3" t="s">
+        <v>998</v>
+      </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
@@ -12424,7 +12670,9 @@
       <c r="Q8" s="3" t="s">
         <v>537</v>
       </c>
-      <c r="R8" s="3"/>
+      <c r="R8" s="3" t="s">
+        <v>999</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -12478,7 +12726,9 @@
       <c r="Q9" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="R9" s="3"/>
+      <c r="R9" s="3" t="s">
+        <v>1000</v>
+      </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -12532,7 +12782,9 @@
       <c r="Q10" s="3" t="s">
         <v>555</v>
       </c>
-      <c r="R10" s="3"/>
+      <c r="R10" s="3" t="s">
+        <v>1001</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -12586,7 +12838,9 @@
       <c r="Q11" s="3" t="s">
         <v>584</v>
       </c>
-      <c r="R11" s="3"/>
+      <c r="R11" s="3" t="s">
+        <v>1002</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
@@ -12640,7 +12894,9 @@
       <c r="Q12" s="3" t="s">
         <v>600</v>
       </c>
-      <c r="R12" s="3"/>
+      <c r="R12" s="3" t="s">
+        <v>1003</v>
+      </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -12694,7 +12950,9 @@
       <c r="Q13" s="3" t="s">
         <v>616</v>
       </c>
-      <c r="R13" s="3"/>
+      <c r="R13" s="3" t="s">
+        <v>1004</v>
+      </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
@@ -12748,7 +13006,9 @@
       <c r="Q14" s="3" t="s">
         <v>632</v>
       </c>
-      <c r="R14" s="3"/>
+      <c r="R14" s="3" t="s">
+        <v>1005</v>
+      </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -12802,7 +13062,9 @@
       <c r="Q15" s="3" t="s">
         <v>648</v>
       </c>
-      <c r="R15" s="3"/>
+      <c r="R15" s="3" t="s">
+        <v>1006</v>
+      </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
@@ -12856,7 +13118,9 @@
       <c r="Q16" s="3" t="s">
         <v>664</v>
       </c>
-      <c r="R16" s="3"/>
+      <c r="R16" s="3" t="s">
+        <v>1007</v>
+      </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
@@ -12910,7 +13174,9 @@
       <c r="Q17" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="R17" s="3"/>
+      <c r="R17" s="3" t="s">
+        <v>1008</v>
+      </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
@@ -12964,7 +13230,9 @@
       <c r="Q18" s="3" t="s">
         <v>696</v>
       </c>
-      <c r="R18" s="3"/>
+      <c r="R18" s="3" t="s">
+        <v>1009</v>
+      </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
@@ -13018,7 +13286,9 @@
       <c r="Q19" s="3" t="s">
         <v>711</v>
       </c>
-      <c r="R19" s="3"/>
+      <c r="R19" s="3" t="s">
+        <v>1010</v>
+      </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
@@ -13072,7 +13342,9 @@
       <c r="Q20" s="3" t="s">
         <v>727</v>
       </c>
-      <c r="R20" s="3"/>
+      <c r="R20" s="3" t="s">
+        <v>1011</v>
+      </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
@@ -13126,7 +13398,9 @@
       <c r="Q21" s="3" t="s">
         <v>743</v>
       </c>
-      <c r="R21" s="3"/>
+      <c r="R21" s="3" t="s">
+        <v>1012</v>
+      </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
@@ -13180,7 +13454,9 @@
       <c r="Q22" s="3" t="s">
         <v>759</v>
       </c>
-      <c r="R22" s="3"/>
+      <c r="R22" s="3" t="s">
+        <v>1013</v>
+      </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
@@ -13234,7 +13510,9 @@
       <c r="Q23" s="3" t="s">
         <v>775</v>
       </c>
-      <c r="R23" s="3"/>
+      <c r="R23" s="3" t="s">
+        <v>1014</v>
+      </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
@@ -13288,7 +13566,9 @@
       <c r="Q24" s="3" t="s">
         <v>791</v>
       </c>
-      <c r="R24" s="3"/>
+      <c r="R24" s="3" t="s">
+        <v>1015</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13297,7 +13577,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
@@ -13772,6 +14052,29 @@
       </c>
       <c r="G18" t="s">
         <v>963</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>992</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1017</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1018</v>
+      </c>
+      <c r="E19">
+        <v>100000000</v>
+      </c>
+      <c r="F19" s="7">
+        <v>300000000</v>
+      </c>
+      <c r="G19" t="s">
+        <v>1019</v>
       </c>
     </row>
   </sheetData>

</xml_diff>